<commit_message>
Plotting enhancements. Frequency tuning of oscillators is succesful.
</commit_message>
<xml_diff>
--- a/apps_Maurice_MAK_REINFORCE/oscillators_freq_3species_6rxns/oscillators_freq_3species_6rxns_MAK_REINFORCE.xlsx
+++ b/apps_Maurice_MAK_REINFORCE/oscillators_freq_3species_6rxns/oscillators_freq_3species_6rxns_MAK_REINFORCE.xlsx
@@ -10,14 +10,14 @@
     <sheet r:id="rId1" sheetId="1" name="Data"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Data'!$A$1:$Y$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Data'!$A$1:$Y$14</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="75">
   <si>
     <t>Timestamp</t>
   </si>
@@ -214,7 +214,34 @@
     <t>https://www.comet.com/maurice-filo/oscillators-freq-3species-6rxns-mak-reinforce/ee34b6d3c7e545afa280ddc572c79e98</t>
   </si>
   <si>
-    <t xml:space="preserve">Reset the risk to 0.9, increased the number of epochs significantly. </t>
+    <t xml:space="preserve">run-10. Reset the risk to 0.9, increased the number of epochs significantly. </t>
+  </si>
+  <si>
+    <t>2026-01-14 10:55:31</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-freq-3species-6rxns-mak-reinforce/4101c46cb3924ad3bc14a856d329b66b</t>
+  </si>
+  <si>
+    <t>run-11. Same conditions as before. Seems to be okay.</t>
+  </si>
+  <si>
+    <t>2026-01-14 16:39:34</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-freq-3species-6rxns-mak-reinforce/1e1f29e5a15344a985442749f7202f91</t>
+  </si>
+  <si>
+    <t>run-12. Same conditions as before. Seems to be good.</t>
+  </si>
+  <si>
+    <t>2026-01-15 06:13:47</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-freq-3species-6rxns-mak-reinforce/6d739bf216564982aa78ea4c1a11a32a</t>
+  </si>
+  <si>
+    <t>run-13. Same conditions as before.</t>
   </si>
 </sst>
 </file>
@@ -589,7 +616,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:Y11"/>
+  <dimension ref="A1:Y14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="4" width="20.005" customWidth="1" bestFit="1"/>
@@ -619,7 +646,7 @@
     <col min="25" max="25" style="4" width="5.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -696,7 +723,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
@@ -765,7 +792,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1" t="s">
         <v>35</v>
       </c>
@@ -834,7 +861,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
         <v>38</v>
       </c>
@@ -905,7 +932,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1" t="s">
         <v>42</v>
       </c>
@@ -976,7 +1003,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
         <v>45</v>
       </c>
@@ -1047,7 +1074,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
         <v>49</v>
       </c>
@@ -1118,7 +1145,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="1" t="s">
         <v>53</v>
       </c>
@@ -1189,7 +1216,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1" t="s">
         <v>56</v>
       </c>
@@ -1260,7 +1287,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="1" t="s">
         <v>59</v>
       </c>
@@ -1331,7 +1358,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="1" t="s">
         <v>63</v>
       </c>
@@ -1350,43 +1377,43 @@
       <c r="H11" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="2">
         <v>3000</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="K11" s="3">
+      <c r="K11" s="2">
         <v>5</v>
       </c>
-      <c r="L11" s="3">
+      <c r="L11" s="2">
         <v>1024</v>
       </c>
-      <c r="M11" s="3">
+      <c r="M11" s="2">
         <v>10240</v>
       </c>
-      <c r="N11" s="3">
+      <c r="N11" s="2">
         <v>128</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P11" s="3">
+      <c r="P11" s="2">
         <v>50</v>
       </c>
-      <c r="Q11" s="3">
-        <v>30</v>
-      </c>
-      <c r="R11" s="3">
+      <c r="Q11" s="2">
+        <v>30</v>
+      </c>
+      <c r="R11" s="2">
         <v>100</v>
       </c>
-      <c r="S11" s="3">
+      <c r="S11" s="2">
         <v>1000</v>
       </c>
-      <c r="T11" s="3">
+      <c r="T11" s="2">
         <v>1</v>
       </c>
-      <c r="U11" s="3">
+      <c r="U11" s="2">
         <v>3</v>
       </c>
       <c r="V11" s="1" t="s">
@@ -1399,6 +1426,219 @@
         <v>37</v>
       </c>
       <c r="Y11" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I12" s="2">
+        <v>1000</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K12" s="2">
+        <v>5</v>
+      </c>
+      <c r="L12" s="2">
+        <v>1024</v>
+      </c>
+      <c r="M12" s="2">
+        <v>10240</v>
+      </c>
+      <c r="N12" s="2">
+        <v>128</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="P12" s="2">
+        <v>50</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>30</v>
+      </c>
+      <c r="R12" s="2">
+        <v>100</v>
+      </c>
+      <c r="S12" s="2">
+        <v>1000</v>
+      </c>
+      <c r="T12" s="2">
+        <v>1</v>
+      </c>
+      <c r="U12" s="2">
+        <v>3</v>
+      </c>
+      <c r="V12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="W12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="X12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y12" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="A13" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I13" s="2">
+        <v>1000</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K13" s="2">
+        <v>5</v>
+      </c>
+      <c r="L13" s="2">
+        <v>1024</v>
+      </c>
+      <c r="M13" s="2">
+        <v>10240</v>
+      </c>
+      <c r="N13" s="2">
+        <v>128</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="P13" s="2">
+        <v>50</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>30</v>
+      </c>
+      <c r="R13" s="2">
+        <v>100</v>
+      </c>
+      <c r="S13" s="2">
+        <v>1000</v>
+      </c>
+      <c r="T13" s="2">
+        <v>1</v>
+      </c>
+      <c r="U13" s="2">
+        <v>3</v>
+      </c>
+      <c r="V13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="W13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="X13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y13" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18">
+      <c r="A14" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I14" s="3">
+        <v>1000</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K14" s="3">
+        <v>5</v>
+      </c>
+      <c r="L14" s="3">
+        <v>1024</v>
+      </c>
+      <c r="M14" s="3">
+        <v>10240</v>
+      </c>
+      <c r="N14" s="3">
+        <v>128</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="P14" s="3">
+        <v>50</v>
+      </c>
+      <c r="Q14" s="3">
+        <v>30</v>
+      </c>
+      <c r="R14" s="3">
+        <v>100</v>
+      </c>
+      <c r="S14" s="3">
+        <v>1000</v>
+      </c>
+      <c r="T14" s="3">
+        <v>1</v>
+      </c>
+      <c r="U14" s="3">
+        <v>3</v>
+      </c>
+      <c r="V14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="W14" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="X14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y14" s="1" t="s">
         <v>34</v>
       </c>
     </row>

</xml_diff>